<commit_message>
docs: link feedback iteration to release commit
</commit_message>
<xml_diff>
--- a/docs/level-5-user-feedback.xlsx
+++ b/docs/level-5-user-feedback.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedback Responses" sheetId="1" r:id="R9f42790c89bf42c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interaction Log" sheetId="2" r:id="Rcb6abe4163894560"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis" sheetId="3" r:id="R50c3f2373d444049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedback Responses" sheetId="1" r:id="Ra169579a1693487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interaction Log" sheetId="2" r:id="R0e8a4646d5ea453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis" sheetId="3" r:id="R88654cf25d9a4a4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -403,7 +403,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb8f0eb97e404645"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R28f9cf8da1554771"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2794,14 +2794,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34.439998626708984" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="16.110000610351562" hidden="0" customWidth="1"/>
@@ -3102,15 +3102,31 @@
       <x:c r="L14" s="30"/>
       <x:c r="M14" s="30"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="31"/>
-      <x:c r="B15" s="36"/>
-      <x:c r="C15" s="36"/>
-      <x:c r="D15" s="36"/>
-      <x:c r="E15" s="36"/>
-      <x:c r="F15" s="36"/>
-      <x:c r="G15" s="36"/>
-      <x:c r="H15" s="32"/>
+    <x:row r="15" ht="61.5" customHeight="1">
+      <x:c r="A15" s="31" t="str">
+        <x:v>Onboarding clarity and proof</x:v>
+      </x:c>
+      <x:c r="B15" s="36" t="str">
+        <x:v>Prior reviewer feedback</x:v>
+      </x:c>
+      <x:c r="C15" s="36" t="str">
+        <x:v>Ship watch-only access and Activity Proof</x:v>
+      </x:c>
+      <x:c r="D15" s="36" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E15" s="36" t="str">
+        <x:v>Om12345-ingle</x:v>
+      </x:c>
+      <x:c r="F15" s="36" t="str">
+        <x:v>Released</x:v>
+      </x:c>
+      <x:c r="G15" s="36" t="str">
+        <x:v>https://github.com/Om12345-ingle/ai-wallet-manager/commit/e86dd17</x:v>
+      </x:c>
+      <x:c r="H15" s="32" t="str">
+        <x:v>Validate again during the genuine 50-wallet study</x:v>
+      </x:c>
       <x:c r="I15" s="30"/>
       <x:c r="J15" s="30"/>
       <x:c r="K15" s="30"/>
@@ -3266,6 +3282,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe8125f97aef46af"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radee7425512a47ad"/>
 </x:worksheet>
 </file>
</xml_diff>